<commit_message>
import clients now work again
</commit_message>
<xml_diff>
--- a/public/files/importTemplate.xlsx
+++ b/public/files/importTemplate.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="105" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{885DE022-C8CF-4C9C-B79D-255F0F2113BD}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ClientBase\client-base\public\files\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF059F8D-F236-4215-9408-8806B102E0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,20 +33,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
-  <si>
-    <t>First</t>
-  </si>
-  <si>
-    <t>Last</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Company</t>
   </si>
   <si>
-    <t>Email</t>
-  </si>
-  <si>
     <t>Phone</t>
   </si>
   <si>
@@ -57,44 +53,44 @@
     <t>Postcode</t>
   </si>
   <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t>ReminderDate</t>
-  </si>
-  <si>
     <t>Test</t>
   </si>
   <si>
-    <t>Subject</t>
-  </si>
-  <si>
-    <t>ClientBase</t>
-  </si>
-  <si>
     <t>t.s@ClientBaseApp.com</t>
   </si>
   <si>
-    <t>021 456 7891</t>
-  </si>
-  <si>
     <t>15 Main rd</t>
   </si>
   <si>
-    <t>Burnside</t>
-  </si>
-  <si>
-    <t>Christchurch</t>
-  </si>
-  <si>
     <t>04-Feb-2022</t>
+  </si>
+  <si>
+    <t>Full name</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Clientbase</t>
+  </si>
+  <si>
+    <t>Email address</t>
+  </si>
+  <si>
+    <t>Reminder date</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Somewhere</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,10 +165,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -195,7 +191,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -483,7 +479,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -491,53 +487,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:U14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.140625" customWidth="1"/>
+    <col min="10" max="12" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
@@ -548,75 +543,74 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-    </row>
-    <row r="2" spans="1:22">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>123456789</v>
+      </c>
+      <c r="C2">
+        <v>123456789</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
       <c r="I2">
-        <v>8053</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:22">
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:22">
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:22">
-      <c r="K7" s="3"/>
-    </row>
-    <row r="8" spans="1:22">
-      <c r="K8" s="3"/>
-    </row>
-    <row r="9" spans="1:22">
-      <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:22">
-      <c r="K10" s="3"/>
-    </row>
-    <row r="11" spans="1:22">
-      <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:22">
-      <c r="K12" s="3"/>
-    </row>
-    <row r="13" spans="1:22">
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:22">
-      <c r="K14" s="3"/>
+        <v>1111</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J3" s="4"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J12" s="3"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="J14" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>